<commit_message>
feat: restore Redis-based presence (pro plan) + faster poll intervals
- Presence API back on Redis: presence:{userId} (5m TTL) + lastseen:{userId} (30d TTL), batched with MGET
- ChatView presence poll restored to 60s (was 180s)
- PresenceIndicator poll restored to 60s (was 180s)
- QA checklist update
</commit_message>
<xml_diff>
--- a/Nexus_QA_Checklist.xlsx
+++ b/Nexus_QA_Checklist.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drive" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Navigation" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HR &amp; Mentor" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,6 +67,9 @@
       <name val="Arial"/>
       <color rgb="005f6368"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -132,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -164,6 +168,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5993,4 +5998,652 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>How to test</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>Expected result</t>
+        </is>
+      </c>
+      <c r="E1" s="15" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="15" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>My HR page</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Open /hr as any role</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Leave balances, request form, holidays, documents, onboarding visible</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Leave request</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Submit annual leave with valid dates</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Request created, appears as pending; managers get notification</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Leave balance guard</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Request more days than remaining allowance</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>400 error with 'insufficient balance' toast</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Leave overlap guard</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Submit a second request overlapping the first</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>409 'overlaps existing request'</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Leave approval</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Admin /admin/hr?tab=leave → Approve</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Status APPROVED; requester notified; balance reduces</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Leave rejection</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Reject with a note</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Status REJECTED, note visible to requester on /hr</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cancel leave</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Requester cancels own pending request</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Status CANCELLED</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Holidays</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Admin adds a holiday; request leave spanning it</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Holiday excluded from working-day count</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HR dashboard</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Open /admin/hr Dashboard tab</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Headcounts, pending leave, on-leave-today, dept chart render</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HR documents (admin)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>People tab → expand person → upload contract</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Doc listed with category; download returns file via signed URL</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HR documents (self)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Upload own doc on /hr; try downloading another user's doc id</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Own doc works; foreign doc returns 403</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Onboarding template</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Expand person → Apply default checklist</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>7 items created; toggling marks complete; progress shows on user's /hr</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Org chart</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Set reporting managers in People, open Org chart tab</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Tree renders with reports nested under managers</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Access control</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Open /admin/hr as CEO (non-admin mgmt) and as DEVELOPER</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CEO can access; DEVELOPER gets 403</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Mentor</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Overview dashboard</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Open /mentor as mentor</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Cohort stats + leaderboard; clicking intern opens profile</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mentor</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Intern profile</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Interns tab → open an intern</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Header stats, submissions, quiz history load</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Mentor</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Mentor assignment</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Assign a mentor from profile dropdown</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Saved; intern notified; shows on roster card</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Mentor</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Evaluation</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Evaluate button → set rubric scores → save</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Overall auto-computed /5; intern notified; visible in intern hub Progress</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Mentor</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1:1 note privacy</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Add note with 'Share with intern' off, then one with it on</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Intern sees only the shared note in Progress tab</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Mentor</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Issue certificate</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Certificates → Issue with grade</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Serial CS-YYYY-XXXXXX generated; intern notified</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Intern</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>My growth panel</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>As intern open Intern Hub → Progress</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Evaluations, shared notes, certificates sections appear</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Intern</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Certificate print</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Click Print / PDF on a certificate</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Printable landscape certificate opens with name, serial, grade</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: DocumentVersion, note tags column, doc presence, PPTX import
Schema: Note gains a queryable `tags String[]` column (was buried in
content JSON), plus a new `DocumentVersion` model for server-persisted
version history shared across Notes, Docs, Sheets and Slides.

APIs: /api/documents/[id]/versions (list/create), /versions/restore,
/api/documents/[id]/presence — real-time collaborator awareness.

Components: DocVersionHistory panel, DocPresenceBar, AppLink wrapper,
note-tags lib (extract legacy tags from content blob).

Libs: cookie-options (shared SameSite/Secure config), doc-access
(permission check helper), docx-export, pptx-import, subdomains,
use-doc-presence hook.

Auth routes: unified cookie options via cookie-options.ts.
Middleware: subdomain routing support.
NotesView/DocsView/SheetsEditor/SlidesEditor: hook into new APIs.
</commit_message>
<xml_diff>
--- a/Nexus_QA_Checklist.xlsx
+++ b/Nexus_QA_Checklist.xlsx
@@ -72,7 +72,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -109,8 +109,13 @@
         <fgColor rgb="00fef9e0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3A3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -132,11 +137,25 @@
         <color rgb="00E8EAED"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D8D7D2"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D8D7D2"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D8D7D2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D8D7D2"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -169,6 +188,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -535,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -557,9 +582,10 @@
           <t>App</t>
         </is>
       </c>
-      <c r="B2" s="3">
-        <f>COUNTIF(Docs!E:E,"Pass")+COUNTIF(Sheets!E:E,"Pass")+COUNTIF(Slides!E:E,"Pass")+COUNTIF(Notes!E:E,"Pass")+COUNTIF(Drive!E:E,"Pass")+COUNTIF(Navigation!E:E,"Pass")</f>
-        <v/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
@@ -579,7 +605,7 @@
         </is>
       </c>
       <c r="B3" s="6">
-        <f>COUNTIF(Docs!E:E,"Fail")+COUNTIF(Sheets!E:E,"Fail")+COUNTIF(Slides!E:E,"Fail")+COUNTIF(Notes!E:E,"Fail")+COUNTIF(Drive!E:E,"Fail")+COUNTIF(Navigation!E:E,"Fail")</f>
+        <f>COUNTIF(Sheets!E2:E300,"Pass")</f>
         <v/>
       </c>
       <c r="C3" s="7">
@@ -687,21 +713,40 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HR &amp; Mentor</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>COUNTIF('HR &amp; Mentor'!E2:E300,"Pass")</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>COUNTIF('HR &amp; Mentor'!E2:E300,"Fail")</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>COUNTA('HR &amp; Mentor'!A2:A300)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9">
-        <f>SUM(B3:B8)</f>
+      <c r="B10">
+        <f>SUM(B3:B9)</f>
         <v/>
       </c>
-      <c r="C9">
-        <f>SUM(C3:C8)</f>
+      <c r="C10">
+        <f>SUM(C3:C9)</f>
         <v/>
       </c>
-      <c r="D9">
-        <f>SUM(D3:D8)</f>
+      <c r="D10">
+        <f>SUM(D3:D9)</f>
         <v/>
       </c>
     </row>
@@ -720,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2115,9 +2160,298 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>Live co-editor presence</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>Open the same sheet in two browsers as two users</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>Avatar stack appears top-right; each shows the other's name</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F54" s="16" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>Remote cell cursor</t>
+        </is>
+      </c>
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>In browser B click cell D5; watch browser A</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Coloured outline + name tag appears on D5 within ~5s</t>
+        </is>
+      </c>
+      <c r="E55" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F55" s="16" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>Cursor is sheet-scoped</t>
+        </is>
+      </c>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>In browser B switch to Sheet2 while A stays on Sheet1</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Remote cursor disappears from A's Sheet1</t>
+        </is>
+      </c>
+      <c r="E56" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>Presence clears on close</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>Close browser B's tab</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Avatar disappears from A within ~15s</t>
+        </is>
+      </c>
+      <c r="E57" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F57" s="16" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>Version history opens</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>Click the clock icon in the header</t>
+        </is>
+      </c>
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>Right panel lists versions with author + timestamp</t>
+        </is>
+      </c>
+      <c r="E58" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F58" s="16" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B59" s="16" t="inlineStr">
+        <is>
+          <t>Auto version on edit</t>
+        </is>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>Type in a cell, wait ~2s, open version history</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>An 'Auto-save' entry exists</t>
+        </is>
+      </c>
+      <c r="E59" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F59" s="16" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>Auto-saves coalesce</t>
+        </is>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>Make 5 edits within a minute; reopen history</t>
+        </is>
+      </c>
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>Only ONE Auto-save row, not five</t>
+        </is>
+      </c>
+      <c r="E60" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>Manual save version</t>
+        </is>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>Click the save icon inside the history panel</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>A 'Manual save' row is added</t>
+        </is>
+      </c>
+      <c r="E61" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F61" s="16" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>Restore a version</t>
+        </is>
+      </c>
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>Edit cells, then Restore an earlier version</t>
+        </is>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>Grid reverts; a 'Before restore' row is created</t>
+        </is>
+      </c>
+      <c r="E62" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F62" s="16" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>Restore is reversible</t>
+        </is>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>After restoring, restore the 'Before restore' entry</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>Returns to the pre-restore state</t>
+        </is>
+      </c>
+      <c r="E63" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="B64" s="16" t="inlineStr">
+        <is>
+          <t>Delete a version</t>
+        </is>
+      </c>
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>Hover a version, click the trash icon</t>
+        </is>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>Row disappears and does not return on reload</t>
+        </is>
+      </c>
+      <c r="E64" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F64" s="16" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2132,7 +2466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3166,9 +3500,272 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>PPTX import - real parse</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>Import a real .pptx made in PowerPoint</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>Slides appear with actual text, not a placeholder</t>
+        </is>
+      </c>
+      <c r="E40" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="16" t="inlineStr">
+        <is>
+          <t>PPTX import - positions</t>
+        </is>
+      </c>
+      <c r="C41" s="16" t="inlineStr">
+        <is>
+          <t>Compare imported slide against the original</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>Text boxes land in roughly the same positions</t>
+        </is>
+      </c>
+      <c r="E41" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F41" s="16" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>PPTX import - images</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>Import a deck containing photos</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>Images render on the imported slides</t>
+        </is>
+      </c>
+      <c r="E42" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F42" s="16" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>PPTX import - tables</t>
+        </is>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>Import a deck containing a table</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>Table appears with its rows and columns</t>
+        </is>
+      </c>
+      <c r="E43" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F43" s="16" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>PPTX import - notes</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>Import a deck with speaker notes; open the notes panel</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>Speaker notes carried across</t>
+        </is>
+      </c>
+      <c r="E44" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>PPTX import is additive</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>Import into a deck that already has slides</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Existing slides kept; imported ones appended</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>PPTX import - bad file</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>Try importing a .txt renamed to .pptx</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>Clear error toast; editor not broken</t>
+        </is>
+      </c>
+      <c r="E46" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>Live co-editor presence</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>Open the same deck as two users</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>Avatar stack shows the other editor</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F47" s="16" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>Peer slide indicator</t>
+        </is>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>Hover a peer's avatar while they view slide 3</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>Tooltip reads 'Name - Slide 3'</t>
+        </is>
+      </c>
+      <c r="E48" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F48" s="16" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>Version history + restore</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>Edit, open history, restore an earlier version</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>Deck reverts; 'Before restore' row created</t>
+        </is>
+      </c>
+      <c r="E49" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F49" s="16" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E40 E41 E42 E43 E44 E45 E46 E47 E48 E49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3183,7 +3780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4328,9 +4925,324 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>Export to Word (.docx)</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>Export menu &gt; Microsoft Word (.docx)</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>File downloads and OPENS in Word without a repair warning</t>
+        </is>
+      </c>
+      <c r="E44" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>DOCX keeps headings</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>Export a doc with H1/H2/H3, open in Word</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Heading styles preserved, not flattened to body text</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>DOCX keeps bold/italic</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>Export text with bold, italic, underline</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>Formatting preserved in Word</t>
+        </is>
+      </c>
+      <c r="E46" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>DOCX keeps lists</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>Export bulleted and numbered lists incl. nesting</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>Lists render as real Word lists</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F47" s="16" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>DOCX keeps tables</t>
+        </is>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>Export a doc containing a table</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>Table renders with borders in Word</t>
+        </is>
+      </c>
+      <c r="E48" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F48" s="16" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>DOCX keeps links</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>Export a doc with a hyperlink</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>Link is clickable in Word</t>
+        </is>
+      </c>
+      <c r="E49" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F49" s="16" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>DOCX keeps images</t>
+        </is>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>Insert an uploaded image, export, open in Word</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>Image embedded in the .docx</t>
+        </is>
+      </c>
+      <c r="E50" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B51" s="16" t="inlineStr">
+        <is>
+          <t>Import Word (.docx)</t>
+        </is>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>Export menu &gt; Import Word (.docx)</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>Content appended into the editor</t>
+        </is>
+      </c>
+      <c r="E51" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F51" s="16" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>Import names untitled doc</t>
+        </is>
+      </c>
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>Import into an Untitled document</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>Doc title becomes the filename</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F52" s="16" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B53" s="16" t="inlineStr">
+        <is>
+          <t>Import is additive</t>
+        </is>
+      </c>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>Import into a doc with existing text</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>Existing text kept, imported content appended</t>
+        </is>
+      </c>
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F53" s="16" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>Versions are server-side</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>Save a version, then open the doc in a different browser</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>Same version list appears (was localStorage-only before)</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F54" s="16" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>Version restore</t>
+        </is>
+      </c>
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>Restore an older version</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Editor reloads it; 'Before restore' row created</t>
+        </is>
+      </c>
+      <c r="E55" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F55" s="16" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4345,7 +5257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4960,9 +5872,272 @@
       </c>
       <c r="F23" s="10" t="inlineStr"/>
     </row>
+    <row r="24">
+      <c r="A24" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>Add a tag</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Select a note, type in the tag field, press Enter</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Chip appears; persists after reload</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Comma commits a tag</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Type 'roadmap,' in the tag field</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Tag commits on the comma</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>Backspace removes a tag</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>With the tag input empty, press Backspace</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>Last chip is removed</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Remove a tag with X</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Click the X on a tag chip</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Chip removed; persists after reload</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>Tags are normalised</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Add '#My Tag' and then 'my-tag'</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>Both become 'my-tag'; the duplicate is rejected</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F28" s="16" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>Duplicate tag rejected</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>Add a tag the note already has</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>Info toast; no duplicate chip</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F29" s="16" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>Tag limit enforced</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>Try to add more than 20 tags</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>Error toast at the limit</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>Sidebar tag list</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Add tags across several notes</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Tags section lists them all</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>Filter by tag</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>Click a tag in the sidebar</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>Only notes with that tag are listed</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F32" s="16" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>Legacy tags still show</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>Open a note tagged before the migration</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>Its old tags still render</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F33" s="16" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E24 E25 E26 E27 E28 E29 E30 E31 E32 E33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5479,7 +6654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5990,9 +7165,324 @@
       </c>
       <c r="F19" s="10" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>docs subdomain</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Visit docs.cybersage.uk</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Documents list loads (same as nexus.../docs)</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>sheets short URL</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Visit docs.cybersage.uk/sheets</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Sheets list loads</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>slides short URL</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Visit docs.cybersage.uk/slides/&lt;id&gt;</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>That presentation opens</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>drive subdomain</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Visit drive.cybersage.uk</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Drive loads</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>meet subdomain</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Visit meet.cybersage.uk/&lt;roomId&gt;</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>That meeting room opens</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Single sign-on across hosts</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Log in on nexus, then open docs.cybersage.uk</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Already authenticated - no login prompt</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>Sidebar crosses subdomain</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>From nexus inbox, click Docs in the sidebar</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>Browser lands on docs.cybersage.uk</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Docs to Sheets stays fast</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>On docs.cybersage.uk, click Sheets</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Client-side nav, no full page reload</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>Hub still serves apps</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Visit nexus.cybersage.uk/docs</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>Still works - old links unbroken</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F28" s="16" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>Deep link after login</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>Logged out, open docs.cybersage.uk/sheets/&lt;id&gt;</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>After login you land on that sheet</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F29" s="16" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>Logout clears all hosts</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>Log out, then visit drive.cybersage.uk</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>Redirected to login</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>API calls same-origin</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>On docs.cybersage.uk open devtools Network</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>/api/* requests return 200, not 404</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: office suite — version history, recent items, comments, goal seek, a11y
Schema: RecentItem model (per-user last-opened tracking for Drive, Docs,
Sheets, Slides); migration at prisma/migrations/20260801_*.

APIs: /api/recent, /api/documents/[id]/comments, /api/documents/[id]/range.

Components: RecentStrip, DocComments, GoalSeekDialog, LinkedRange,
ConflictBanner, AccessibilityPanel, ShortcutHelp.

Sheets: expanded formula engine (512-line formula.ts overhaul), goal-seek
solver, cross-app linked ranges, conflict detection.

Libs: use-recent, use-voice-typing, doc-conflict, doc-comment-notify,
doc-to-slides, goal-seek, a11y-check, docx-export improvements.

Docs/verification walkthroughs and office-suite gap analysis added.
</commit_message>
<xml_diff>
--- a/Nexus_QA_Checklist.xlsx
+++ b/Nexus_QA_Checklist.xlsx
@@ -765,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2446,12 +2446,148 @@
       </c>
       <c r="F64" s="16" t="n"/>
     </row>
+    <row r="65">
+      <c r="A65" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B65" s="16" t="inlineStr">
+        <is>
+          <t>Cell comments</t>
+        </is>
+      </c>
+      <c r="C65" s="16" t="inlineStr">
+        <is>
+          <t>Select B7, open Comments, post</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>Thread is tagged B7</t>
+        </is>
+      </c>
+      <c r="E65" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F65" s="16" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B66" s="16" t="inlineStr">
+        <is>
+          <t>Jump to commented cell</t>
+        </is>
+      </c>
+      <c r="C66" s="16" t="inlineStr">
+        <is>
+          <t>Click the B7 chip on a thread</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>Selection moves to B7</t>
+        </is>
+      </c>
+      <c r="E66" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F66" s="16" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>Cross-sheet comment chip</t>
+        </is>
+      </c>
+      <c r="C67" s="16" t="inlineStr">
+        <is>
+          <t>Comment on Sheet2, view from Sheet1</t>
+        </is>
+      </c>
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>Chip reads 'Sheet2!&lt;cell&gt;'</t>
+        </is>
+      </c>
+      <c r="E67" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F67" s="16" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B68" s="16" t="inlineStr">
+        <is>
+          <t>Recent strip</t>
+        </is>
+      </c>
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>Open a few sheets, return to the Sheets list</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>Recent row shows them, most recent first</t>
+        </is>
+      </c>
+      <c r="E68" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F68" s="16" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>Conflict detected</t>
+        </is>
+      </c>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>Two browsers, save in B then edit in A</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>Conflict banner appears; no silent data loss</t>
+        </is>
+      </c>
+      <c r="E69" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
     <dataValidation sqref="E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E65 E66 E67 E68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2466,7 +2602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3760,12 +3896,148 @@
       </c>
       <c r="F49" s="16" t="n"/>
     </row>
+    <row r="50">
+      <c r="A50" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>Slide comments</t>
+        </is>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>Open slide 3, post a comment</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>Thread tagged 'Slide 3'</t>
+        </is>
+      </c>
+      <c r="E50" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B51" s="16" t="inlineStr">
+        <is>
+          <t>Jump to commented slide</t>
+        </is>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>Click the Slide 3 chip</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>Editor jumps to slide 3</t>
+        </is>
+      </c>
+      <c r="E51" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F51" s="16" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>Deleted slide handled</t>
+        </is>
+      </c>
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>Comment on a slide, delete it, reopen comments</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>Chip reads '(deleted slide)', no crash</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F52" s="16" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B53" s="16" t="inlineStr">
+        <is>
+          <t>Recent strip</t>
+        </is>
+      </c>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>Open a few decks, return to the Slides list</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>Recent row shows them</t>
+        </is>
+      </c>
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F53" s="16" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>Conflict detected</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>Two browsers, save in B then edit in A</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>Conflict banner appears; no silent data loss</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F54" s="16" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
     <dataValidation sqref="E40 E41 E42 E43 E44 E45 E46 E47 E48 E49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E50 E51 E52 E53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3780,7 +4052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5237,12 +5509,382 @@
       </c>
       <c r="F55" s="16" t="n"/>
     </row>
+    <row r="56">
+      <c r="A56" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>Comments persist</t>
+        </is>
+      </c>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>Add a comment, hard-refresh the page</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Comment is still there (was lost before)</t>
+        </is>
+      </c>
+      <c r="E56" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>Comment shows real author</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>Add a comment</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Your actual name, not 'You'</t>
+        </is>
+      </c>
+      <c r="E57" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F57" s="16" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>Comment anchored to text</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>Select a phrase, then add a comment</t>
+        </is>
+      </c>
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>Composer shows the quoted phrase</t>
+        </is>
+      </c>
+      <c r="E58" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F58" s="16" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B59" s="16" t="inlineStr">
+        <is>
+          <t>Jump to commented text</t>
+        </is>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>Click the text chip on a comment thread</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>Editor scrolls to and selects that text</t>
+        </is>
+      </c>
+      <c r="E59" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F59" s="16" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>Deleted text handled</t>
+        </is>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>Comment on text, delete the text, reopen comments</t>
+        </is>
+      </c>
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>Chip reads '(text removed)', no crash</t>
+        </is>
+      </c>
+      <c r="E60" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>Reply to a thread</t>
+        </is>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>Click Reply, type, press Cmd+Enter</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>Reply nests under the thread</t>
+        </is>
+      </c>
+      <c r="E61" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F61" s="16" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>Resolve a thread</t>
+        </is>
+      </c>
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>Click the tick on a thread</t>
+        </is>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>Thread disappears from the open list</t>
+        </is>
+      </c>
+      <c r="E62" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F62" s="16" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>View resolved</t>
+        </is>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>Click the eye icon</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>Resolved threads are listed</t>
+        </is>
+      </c>
+      <c r="E63" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B64" s="16" t="inlineStr">
+        <is>
+          <t>Mention notifies</t>
+        </is>
+      </c>
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>Comment '@Name' using a real colleague's name</t>
+        </is>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>They get a Mention notification linking to the doc</t>
+        </is>
+      </c>
+      <c r="E64" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F64" s="16" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="B65" s="16" t="inlineStr">
+        <is>
+          <t>Cannot edit others' comments</t>
+        </is>
+      </c>
+      <c r="C65" s="16" t="inlineStr">
+        <is>
+          <t>As user B, try to edit user A's comment</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>Blocked with 403</t>
+        </is>
+      </c>
+      <c r="E65" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F65" s="16" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="B66" s="16" t="inlineStr">
+        <is>
+          <t>Conflict detected</t>
+        </is>
+      </c>
+      <c r="C66" s="16" t="inlineStr">
+        <is>
+          <t>Open the same doc in two browsers, edit and save in B, then type in A</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>A sees 'Someone else edited this' banner instead of silently overwriting</t>
+        </is>
+      </c>
+      <c r="E66" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F66" s="16" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>Reload theirs</t>
+        </is>
+      </c>
+      <c r="C67" s="16" t="inlineStr">
+        <is>
+          <t>On the conflict banner click 'Reload theirs'</t>
+        </is>
+      </c>
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>Editor loads B's version</t>
+        </is>
+      </c>
+      <c r="E67" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F67" s="16" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="B68" s="16" t="inlineStr">
+        <is>
+          <t>Keep mine</t>
+        </is>
+      </c>
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>On the conflict banner click 'Keep mine'</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>A's version saves and wins</t>
+        </is>
+      </c>
+      <c r="E68" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F68" s="16" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>Export opens in Word</t>
+        </is>
+      </c>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>Export &gt; Microsoft Word, open the file in real Word</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>Opens with NO 'needs repair' prompt</t>
+        </is>
+      </c>
+      <c r="E69" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
     <dataValidation sqref="E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E56 E57 E58 E59 E60 E61 E62 E63 E64 E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E66 E67 E68 E69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6152,7 +6794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6637,9 +7279,142 @@
       </c>
       <c r="F18" s="10" t="inlineStr"/>
     </row>
+    <row r="19">
+      <c r="A19" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Office docs listed</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Open Drive root</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Docs/Sheets/Slides appear alongside uploaded files</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Open doc from Drive</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Click a spreadsheet in Drive</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Opens the Sheets editor on docs.cybersage.uk (not a 404)</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>New &gt; spreadsheet</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>New menu &gt; New spreadsheet</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Creates and opens a new sheet</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Recent by open, not edit</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Have a colleague edit a file you never opened; check Recent</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Their file does NOT jump to the top of your Recent</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Recent reflects your opens</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Open a document, go to Drive &gt; Recent</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>It is at the top</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E19 E20 E21 E22 E23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6654,7 +7429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7477,12 +8252,174 @@
       </c>
       <c r="F31" s="16" t="n"/>
     </row>
+    <row r="32">
+      <c r="A32" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>Search crosses subdomains</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>From nexus, search and open a spreadsheet</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>Lands on docs.cybersage.uk, not a 404</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F32" s="16" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>Old comments endpoint gone</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>GET /api/docs/&lt;id&gt;/comments</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>Returns 410, not document data</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F33" s="16" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>Long pages scroll</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>Open Settings, Users, People, Teams, Billing, Compliance, Admin pages</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>Content scrolls to the bottom (was clipped with no scrollbar)</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F34" s="16" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>Paned views unaffected</t>
+        </is>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>Open Inbox, Chat, Drive, Docs</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Each column scrolls on its own; headers stay put</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F35" s="16" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>Mobile heights</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>Open Notes / Meet / Docs on a phone</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>Fills the screen without being cut off behind the tab bar</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F36" s="16" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>Shortcut overlay</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>Press Cmd+/ (Ctrl+/) in Docs, Sheets or Slides</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Keyboard shortcut dialog opens; Esc closes it</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="F37" s="16" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
     <dataValidation sqref="E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E32 E33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E34 E35 E36 E37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not tested,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>